<commit_message>
Add verification worksheet and pipeline, Desktop intake tool; reclass C-1205/C-1206
- 07 Verification_Worksheet.md: procedure, sources, deadlines and fallbacks
  for all 15 BLOCKING claims, 3 low-risk claims and 7 platform facts
- verification_results.csv applied by gen_ledger.py (requires URL, quote,
  date and verifier); outputs regenerate the ledger, schedule and workbook
- tools/desktop_intake.py: read-only local inventory of the Desktop folder
  with reference-video MD5 detection and topic-overlap flags (tested)
- C-1205/C-1206 QUALIFIED from the USFA excerpt in appendix D2 (CL-012)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PDJn9KvK6oMk1DbDggswng
</commit_message>
<xml_diff>
--- a/Worldosphere_Analysis_and_Launch_Plan_2026-10-14/Worldosphere_Launch_Workbook.xlsx
+++ b/Worldosphere_Analysis_and_Launch_Plan_2026-10-14/Worldosphere_Launch_Workbook.xlsx
@@ -32,7 +32,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Pilot hours'!$A$1:$F$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Tracking'!$A$1:$V$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'QA log'!$A$1:$L$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Change log'!$A$1:$E$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Change log'!$A$1:$E$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Asset register'!$A$1:$K$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5898,7 +5898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6238,13 +6238,40 @@
           <t>CL-012</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr"/>
-      <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>C-1205 re-worded to the evidence and re-classed QUALIFIED; C-1206 re-classed QUALIFIED; a verification-results pipeline and worksheet added</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>The USFA escape-planning excerpt already in appendix D2 §3c ("if the door is hot, keep it closed and use your second way out") meets the same evidence standard as other SUPPORTED rows; the "back of the hand" detail had no evidence and was removed</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>ledger, WS-012 brief, calendar, 07 Verification_Worksheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>CL-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E13"/>
+  <autoFilter ref="A1:E14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8186,7 +8213,7 @@
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>C-1201, C-1202, C-1203, C-1204, C-1206 (BLOCKING: window as second way out); C-1205 only if verified</t>
+          <t>C-1201, C-1202, C-1203, C-1204, C-1206 (QUALIFIED: window as second way out); C-1205 (QUALIFIED; heat check only)</t>
         </is>
       </c>
       <c r="S13" s="2" t="inlineStr">
@@ -12166,7 +12193,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>C-1201, C-1202, C-1203, C-1204, C-1206 (BLOCKING: window as second way out); C-1205 only if verified</t>
+          <t>C-1201, C-1202, C-1203, C-1204, C-1206 (QUALIFIED: window as second way out); C-1205 (QUALIFIED; heat check only)</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -24560,7 +24587,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Feel a closed door with the back of your hand before opening</t>
+          <t>Check a closed door for heat before opening it; if it is hot, keep it closed and use the second way out</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -24570,7 +24597,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>NFPA / Red Cross (common guidance; not retrieved)</t>
+          <t>USFA escape-planning pictographs (research appendix D2 §3c, search-excerpt paraphrase: if the door is hot, keep it closed and use your second way out); NFPA escape planning</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -24580,22 +24607,22 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>The earlier 'back of the hand' detail is NOT in the retrieved evidence and must not be scripted unless verified; confirm the live USFA wording (QA F-03)</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>"Back of the hand. Hot? Use the window."</t>
+          <t>"Hot door? Keep it shut. Use your second way out."</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Hand to door</t>
+          <t>Owen's hand near the door, then he turns to the window</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED — BLOCKING if used</t>
+          <t>QUALIFIED</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
@@ -24616,7 +24643,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Plan two ways out of every room; a window can be the second way out when smoke blocks the door route</t>
+          <t>Use a second way out when the door route is blocked; a window can be that second way out</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -24626,7 +24653,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>NFPA home fire escape planning; USFA escape-planning pictographs (pages cited in research appendix D2 §3c; this wording not retrieved)</t>
+          <t>USFA escape-planning pictographs (research appendix D2 §3c, search-excerpt paraphrase: if the door is hot, keep it closed and use your second way out); NFPA home fire escape planning ('two ways out' wording to confirm live)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -24636,12 +24663,12 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Only where the window leads somewhere safe</t>
+          <t>Only where the window leads somewhere safe; confirm the live NFPA/USFA wording before publication (QA F-03)</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>"Every room needs a second way out."</t>
+          <t>"He uses his second way out: the window."</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -24651,7 +24678,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED — BLOCKING</t>
+          <t>QUALIFIED</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Verify all blocking claims and platform facts; revise scripts the evidence contradicted
- verification_results.csv: 18 claims checked against official/primary
  sources (NWS/NOAA, CDC/CPSC, NASA/ESA/AMS, USAP/BAS, MN DNR, NFPA/USFA,
  CAL FIRE, Ready.gov, FCC, peer-reviewed); ledger now has no BLOCKING rows
- WS-002: laminated side glass defeats punch tools, so Owen lowers the
  power window; package regenerated (119 words, 59.6 s)
- WS-020 drops the unsourced transformer hum; WS-025 drops 'Only Rescue';
  WS-028 says 'toward where the crowd thins'; six REAL RULE lines finalised
- Platform facts P1-P7 checked on YouTube Help (Content ID pages conflict,
  conservative rule kept); upload audio 384 kbps
- Docs, schedule, workbook and change log (CL-013) updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PDJn9KvK6oMk1DbDggswng
</commit_message>
<xml_diff>
--- a/Worldosphere_Analysis_and_Launch_Plan_2026-10-14/Worldosphere_Launch_Workbook.xlsx
+++ b/Worldosphere_Analysis_and_Launch_Plan_2026-10-14/Worldosphere_Launch_Workbook.xlsx
@@ -32,7 +32,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Pilot hours'!$A$1:$F$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Tracking'!$A$1:$V$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'QA log'!$A$1:$L$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Change log'!$A$1:$E$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Change log'!$A$1:$E$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Asset register'!$A$1:$K$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5898,7 +5898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6265,13 +6265,40 @@
           <t>CL-013</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr"/>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>All 15 BLOCKING claims verified (9 SUPPORTED, 6 QUALIFIED) and platform facts P1–P7 checked on official pages; WS-002 shows the power window instead of a punch tool; WS-020 drops the transformer-hum claim and says "for hours"; WS-025 title drops "Only Rescue"; WS-028 says "toward where the crowd thins" instead of "diagonally"; six REAL RULE lines finalised; upload audio bitrate 384 kbps</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Official and primary sources found once the search budget reset (verification_results.csv; 23 §2). Laminated side glass defeats punch tools (AAA/NHTSA ESV); the hum, "only rescue" and "diagonal" wordings had no source</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>ledger, calendar, 12 briefs, WS-002 package, 12, 20, 22, 23, 00, 01</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>CL-014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr"/>
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E14"/>
+  <autoFilter ref="A1:E15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7193,7 +7220,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Owen tries the door (pinned by water pressure), switches to the side window with his keyring punch and escapes before the waterline reaches the glass</t>
+          <t>Owen tries the door (pinned by water pressure), lowers the side window with the power switch while the electrics still work, and escapes before the waterline reaches the glass</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -7243,7 +7270,7 @@
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>C-201, C-202, C-203, C-204, C-205 (BLOCKING order check), C-206, C-207</t>
+          <t>C-201, C-202, C-203, C-204, C-205 (QUALIFIED: SWOC order), C-206, C-207 (SUPPORTED: laminated glass; power window shown)</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
@@ -7534,7 +7561,7 @@
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>C-501, C-502, C-503, C-504, C-506 (BLOCKING: fresh air + call for help); C-505 (BLOCKING if alarms mentioned)</t>
+          <t>C-501, C-502, C-503, C-504, C-506 (fresh air + call for help; verified), C-505 (alarms; verified)</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
@@ -8019,7 +8046,7 @@
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>C-1001, C-1002, C-011, C-022, C-501/502; C-1003 must be cut or verified</t>
+          <t>C-1001, C-1002, C-011, C-022, C-501/502; C-1003 (qualified: no hour numbers)</t>
         </is>
       </c>
       <c r="S11" s="2" t="inlineStr">
@@ -8504,7 +8531,7 @@
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>WR-01 (fever, bite), WR-04; C-1501 (no real numbers unless verified)</t>
+          <t>WR-01 (fever, bite), WR-04; C-1501 (verified)</t>
         </is>
       </c>
       <c r="S16" s="2" t="inlineStr">
@@ -8698,7 +8725,7 @@
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>C-1701, C-1702, C-1703; C-1704 not animated unless verified</t>
+          <t>C-1701, C-1702, C-1703, C-1704 (rip signs; verified)</t>
         </is>
       </c>
       <c r="S18" s="2" t="inlineStr">
@@ -8755,7 +8782,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Leonid meteor-shower week brings meteor curiosity [BK]. The script must state that shower meteors are harmless dust (C-1802). Conditional on verifying C-1801.</t>
+          <t>Leonid meteor-shower week brings meteor curiosity [BK]. The script must state that shower meteors are harmless dust (C-1802). C-1801 and C-1802 verified 2026-10-14 (NASA, ESA, AMS).</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -8785,7 +8812,7 @@
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>SAFE — Away from the glass, not toward it. REAL RULE (pending verification): A bright flash in the sky? Stay away from windows.</t>
+          <t>SAFE — Away from the glass, not toward it. REAL RULE: A bright flash in the sky? Stay away from windows.</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr">
@@ -8795,7 +8822,7 @@
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>C-1801 (BLOCKING), C-1802 (BLOCKING)</t>
+          <t>C-1801, C-1802 (both verified)</t>
         </is>
       </c>
       <c r="S19" s="2" t="inlineStr">
@@ -8934,7 +8961,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Frame 0: green aurora over a southern town, people filming; Owen listening to a humming transformer: 'Everyone was filming the sky. Owen was listening to the transformers.'</t>
+          <t>Frame 0: green aurora over a southern town, people filming; Owen, back turned, looking at the power lines: 'Everyone was filming the sky. Owen was watching the power lines.'</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -8949,7 +8976,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>A big-picture P3 in week 3. Conditional on verifying C-2001; swap to R01/R08 if verification fails.</t>
+          <t>A big-picture P3 in week 3. C-2001 is qualified (NOAA SWPC): say the 1989 blackout lasted 'hours', and never state a transformer hum as fact.</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -8989,7 +9016,7 @@
       </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>C-2001 (BLOCKING), C-1001, C-1002</t>
+          <t>C-2001 (qualified: 'for hours'; no transformer-hum claim), C-1001, C-1002</t>
         </is>
       </c>
       <c r="S21" s="2" t="inlineStr">
@@ -9086,7 +9113,7 @@
       </c>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>C-2101, C-2102, C-2103; C-2104 not shown unless verified</t>
+          <t>C-2101, C-2102, C-2103, C-2104 (4 in. new clear ice; verified)</t>
         </is>
       </c>
       <c r="S22" s="2" t="inlineStr">
@@ -9230,7 +9257,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Owen leaves when told rather than when he's ready, and passes the checkpoint before the road closes (pending verified guidance)</t>
+          <t>Owen leaves when told rather than when he's ready, and passes the checkpoint before the road closes (C-2301, verified)</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -9240,7 +9267,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Conditional slot. Wildfire interest is high after recent fires [BK]. It needs verification of C-2301; reserve R01/R02 is ready.</t>
+          <t>Conditional slot. Wildfire interest is high after recent fires [BK]. C-2301 verified (Ready.gov, NFPA, CAL FIRE); reserve R01/R02 stays ready.</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -9270,7 +9297,7 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>ESCAPED — He left when told, not when ready. (REAL RULE pending verification)</t>
+          <t>ESCAPED — He left when told, not when ready. REAL RULE: Wildfire: leave as soon as you're told to. Sooner if you feel unsafe.</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
@@ -9280,7 +9307,7 @@
       </c>
       <c r="R24" s="2" t="inlineStr">
         <is>
-          <t>C-2301 (BLOCKING)</t>
+          <t>C-2301 (verified)</t>
         </is>
       </c>
       <c r="S24" s="2" t="inlineStr">
@@ -9409,7 +9436,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Avalanche: Why Your Friends Are Your Only Rescue</t>
+          <t>Avalanche: Why Your Friends Are the Rescue Team</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -9424,7 +9451,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Tess searches immediately (beacon, probe, shovel) instead of going for help, and finds Jun in time (pending verified guidance)</t>
+          <t>Tess searches immediately (beacon, probe, shovel) instead of going for help, and finds Jun in time (C-2501, qualified)</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -9434,7 +9461,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Ski-season start. Conditional on C-2501 verification; reuses snow assets from Station Zero.</t>
+          <t>Ski-season start. C-2501 qualified (survival-curve research; avalanche.org); reuses snow assets from Station Zero.</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -9464,7 +9491,7 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>SURVIVED — She searched instead of going for help. (REAL RULE pending verification)</t>
+          <t>SURVIVED — She searched instead of going for help. REAL RULE: Avalanche: your partners are the rescue team. Speed is everything.</t>
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr">
@@ -9474,7 +9501,7 @@
       </c>
       <c r="R26" s="2" t="inlineStr">
         <is>
-          <t>C-2501 (BLOCKING)</t>
+          <t>C-2501 (qualified)</t>
         </is>
       </c>
       <c r="S26" s="2" t="inlineStr">
@@ -9628,7 +9655,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>US Thanksgiving. Conditional on verifying C-2701 (NFPA/USFA); reserve R01 is ready.</t>
+          <t>US Thanksgiving. C-2701 verified (USFA, NFPA); reserve R01 stays ready.</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -9658,7 +9685,7 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>SAFE — He cut the heat and smothered it. (REAL RULE pending verification)</t>
+          <t>SAFE — He cut the heat and smothered it. REAL RULE: Grease fire? Never water. Lid on, heat off.</t>
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr">
@@ -9668,7 +9695,7 @@
       </c>
       <c r="R28" s="2" t="inlineStr">
         <is>
-          <t>C-2701 (BLOCKING)</t>
+          <t>C-2701 (verified; NFPA discourages oil fryers)</t>
         </is>
       </c>
       <c r="S28" s="2" t="inlineStr">
@@ -9715,7 +9742,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Tess keeps her feet, protects her chest and moves diagonally with the flow to a gap at the edge (pending verified guidance)</t>
+          <t>Tess keeps her feet, protects her chest and moves with the flow toward where the crowd thins at the edge (C-2801, qualified)</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -9725,7 +9752,7 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Black Friday. Conditional on verifying C-2801 plus a sensitivity review; reserve R02 is ready.</t>
+          <t>Black Friday. C-2801 is qualified (expert guidance); a sensitivity review is still required before script lock; reserve R02 is ready.</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -9755,7 +9782,7 @@
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>SAFE — With the crowd, then out of it. (REAL RULE pending verification)</t>
+          <t>SAFE — With the crowd, then out of it. REAL RULE: Crowd surge? Stay on your feet. Arms up to protect your chest.</t>
         </is>
       </c>
       <c r="Q29" s="2" t="inlineStr">
@@ -9765,7 +9792,7 @@
       </c>
       <c r="R29" s="2" t="inlineStr">
         <is>
-          <t>C-2801 (BLOCKING)</t>
+          <t>C-2801 (qualified; sensitivity review)</t>
         </is>
       </c>
       <c r="S29" s="2" t="inlineStr">
@@ -9822,7 +9849,7 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Winter weekend. A natural bridge to December's winter theme. Conditional on verifying C-2901.</t>
+          <t>Winter weekend. A natural bridge to December's winter theme. C-2901 verified (NWS).</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -9852,7 +9879,7 @@
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>WALK: LOST · WAIT: SURVIVED — Stay with the car. (REAL RULE pending verification)</t>
+          <t>WALK: LOST · WAIT: SURVIVED — Stay with the car. REAL RULE: Stranded in snow? Stay with the car. Keep the tailpipe clear.</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr">
@@ -9862,7 +9889,7 @@
       </c>
       <c r="R30" s="2" t="inlineStr">
         <is>
-          <t>C-2901 (BLOCKING)</t>
+          <t>C-2901 (verified)</t>
         </is>
       </c>
       <c r="S30" s="2" t="inlineStr">
@@ -11443,7 +11470,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>C-201, C-202, C-203, C-204, C-205 (BLOCKING order check), C-206, C-207</t>
+          <t>C-201, C-202, C-203, C-204, C-205 (QUALIFIED: SWOC order), C-206, C-207 (SUPPORTED: laminated glass; power window shown)</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -11668,7 +11695,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>C-501, C-502, C-503, C-504, C-506 (BLOCKING: fresh air + call for help); C-505 (BLOCKING if alarms mentioned)</t>
+          <t>C-501, C-502, C-503, C-504, C-506 (fresh air + call for help; verified), C-505 (alarms; verified)</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -12043,7 +12070,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>C-1001, C-1002, C-011, C-022, C-501/502; C-1003 must be cut or verified</t>
+          <t>C-1001, C-1002, C-011, C-022, C-501/502; C-1003 (qualified: no hour numbers)</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -12418,7 +12445,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>WR-01 (fever, bite), WR-04; C-1501 (no real numbers unless verified)</t>
+          <t>WR-01 (fever, bite), WR-04; C-1501 (verified)</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
@@ -12568,7 +12595,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>C-1701, C-1702, C-1703; C-1704 not animated unless verified</t>
+          <t>C-1701, C-1702, C-1703, C-1704 (rip signs; verified)</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -12623,7 +12650,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>SAFE — Away from the glass, not toward it. REAL RULE (pending verification): A bright flash in the sky? Stay away from windows.</t>
+          <t>SAFE — Away from the glass, not toward it. REAL RULE: A bright flash in the sky? Stay away from windows.</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -12643,7 +12670,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>C-1801 (BLOCKING), C-1802 (BLOCKING)</t>
+          <t>C-1801, C-1802 (both verified)</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
@@ -12793,7 +12820,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>C-2001 (BLOCKING), C-1001, C-1002</t>
+          <t>C-2001 (qualified: 'for hours'; no transformer-hum claim), C-1001, C-1002</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -12868,7 +12895,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>C-2101, C-2102, C-2103; C-2104 not shown unless verified</t>
+          <t>C-2101, C-2102, C-2103, C-2104 (4 in. new clear ice; verified)</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -12998,7 +13025,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>ESCAPED — He left when told, not when ready. (REAL RULE pending verification)</t>
+          <t>ESCAPED — He left when told, not when ready. REAL RULE: Wildfire: leave as soon as you're told to. Sooner if you feel unsafe.</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -13018,7 +13045,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>C-2301 (BLOCKING)</t>
+          <t>C-2301 (verified)</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -13128,7 +13155,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Avalanche: Why Your Friends Are Your Only Rescue</t>
+          <t>Avalanche: Why Your Friends Are the Rescue Team</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -13148,7 +13175,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>SURVIVED — She searched instead of going for help. (REAL RULE pending verification)</t>
+          <t>SURVIVED — She searched instead of going for help. REAL RULE: Avalanche: your partners are the rescue team. Speed is everything.</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -13168,7 +13195,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>C-2501 (BLOCKING)</t>
+          <t>C-2501 (qualified)</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
@@ -13298,7 +13325,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>SAFE — He cut the heat and smothered it. (REAL RULE pending verification)</t>
+          <t>SAFE — He cut the heat and smothered it. REAL RULE: Grease fire? Never water. Lid on, heat off.</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -13318,7 +13345,7 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>C-2701 (BLOCKING)</t>
+          <t>C-2701 (verified; NFPA discourages oil fryers)</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
@@ -13373,7 +13400,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>SAFE — With the crowd, then out of it. (REAL RULE pending verification)</t>
+          <t>SAFE — With the crowd, then out of it. REAL RULE: Crowd surge? Stay on your feet. Arms up to protect your chest.</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -13393,7 +13420,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>C-2801 (BLOCKING)</t>
+          <t>C-2801 (qualified; sensitivity review)</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
@@ -13448,7 +13475,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>WALK: LOST · WAIT: SURVIVED — Stay with the car. (REAL RULE pending verification)</t>
+          <t>WALK: LOST · WAIT: SURVIVED — Stay with the car. REAL RULE: Stranded in snow? Stay with the car. Keep the tailpipe clear.</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -13468,7 +13495,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>C-2901 (BLOCKING)</t>
+          <t>C-2901 (verified)</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
@@ -22315,7 +22342,7 @@
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="35" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
     <col width="34" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
@@ -22749,7 +22776,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>General atmospheric physics (condensation of warm moist breath in cold air). No agency page retrieved this session</t>
+          <t>General atmospheric physics (condensation of warm moist breath in cold air). No agency page retrieved this session · VERIFIED 2026-10-14 by Claude cloud session via official-domain web search (excerpts; confirm live wording at QA F-03): https://www.weather.gov/media/shv/education_resource_library/atmosphere/Atmosphere_AnswerKey.pdf — "As you exhale, the warm, moist air is cooled to the point where the water vapor CONDENSES into a cloud."</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -22759,7 +22786,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Visibility depends on temperature and humidity; no fixed threshold stated</t>
+          <t>No temperature threshold on screen</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -22774,7 +22801,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED (low risk; add one citable source, e.g. a NOAA/NWS or university explainer)</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -23197,7 +23224,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>U. Manitoba lists 'Seatbelts off, Windows open… Out'; CBS (2024) reports Giesbrecht reversed the order — not confirmed</t>
+          <t>U. Manitoba lists 'Seatbelts off, Windows open… Out'; CBS (2024) reports Giesbrecht reversed the order — not confirmed · VERIFIED 2026-10-14 by Claude cloud session via official-domain web search (excerpts; confirm live wording at QA F-03): https://pubmed.ncbi.nlm.nih.gov/20681239/ — "[search excerpt] recommends unfastening seatbelts, opening windows, releasing children from restraints ... then exiting, children first (SWOC: Seatbelts off, Windows open, Out immediately, Children first)"</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -23207,12 +23234,12 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Published SWOC order is seatbelts, then windows (Giesbrecht &amp; McDonald 2010). A 2024 CBS report says the researcher has reversed the order; no primary source confirms it. Recheck the U. Manitoba page at QA F-03; Version B ready</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Script carries Version A and Version B; use the order in the current Giesbrecht/U. Manitoba guidance</t>
+          <t>"Belt off. Window down."</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -23222,7 +23249,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED — BLOCKING</t>
+          <t>QUALIFIED</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -23253,7 +23280,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>McDonald &amp; Giesbrecht 2013 review (Aviat Space Environ Med; PDF via Kids and Cars); Giesbrecht via CBS</t>
+          <t>McDonald &amp; Giesbrecht 2013 review (Aviat Space Environ Med; PDF via Kids and Cars); Giesbrecht via CBS · VERIFIED 2026-10-14 by Claude cloud session via official-domain web search (excerpts; confirm live wording at QA F-03): https://static.nhtsa.gov/esv/pdf/ESV/Proceedings/28/ESV26-243%20FINAL_Corrected%20Manuscript.pdf — "[search excerpt] In AAA testing, none of six window-breaking tools breached laminated glazing, while four broke tempered glass"</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -23263,12 +23290,12 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Some newer vehicles have laminated side glass that tools may not break (UNVERIFIED) — mention in description only</t>
+          <t>Tools break tempered glass only; many newer cars have laminated side glass. Not shown in WS-002; side window, not windshield, still applies</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>"Keep a window tool where you can reach it."</t>
+          <t>"Side window, not the windshield."</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -23309,7 +23336,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>NHTSA / manufacturers (not verified)</t>
+          <t>NHTSA / manufacturers (not verified) · VERIFIED 2026-10-14 by Claude cloud session via official-domain web search (excerpts; confirm live wording at QA F-03): https://static.nhtsa.gov/esv/pdf/ESV/Proceedings/28/ESV26-243%20FINAL_Corrected%20Manuscript.pdf — "[search excerpt] In AAA testing, none of six window-breaking tools breached laminated glazing ... Power can fail early, though most systems last several minutes (also PMC6545703: laminated side glass described as virtually impossible to break)"</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -23319,22 +23346,22 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
+          <t>Open the power window as early as possible while the electrics still work</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>"Window down — while the power still works."</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Not on screen</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED (description caveat only)</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -23813,7 +23840,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>CDC/CPSC (commonly advised; not retrieved this session)</t>
+          <t>CDC/CPSC (commonly advised; not retrieved this session) · VERIFIED 2026-10-14 by Claude cloud session via official-domain web search (excerpts; confirm live wording at QA F-03): https://www.cpsc.gov/safety-education/safety-guides/carbon-monoxide/carbon-monoxide-fact-sheet — "[search excerpt] alarms on every level of the home and outside sleeping areas ... Hardwired or plug-in units should still have battery backup"</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -23838,7 +23865,7 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED — BLOCKING if used</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
@@ -23869,7 +23896,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>CDC / CPSC first-response guidance (07 §4 standard wording; the specific page wording was not retrieved this session)</t>
+          <t>CDC / CPSC first-response guidance (07 §4 standard wording; the specific page wording was not retrieved this session) · VERIFIED 2026-10-14 by Claude cloud session via official-domain web search (excerpts; confirm live wording at QA F-03): https://www.cpsc.gov/Safety-Education/Safety-Education-Centers/Carbon-Monoxide-Information-Center/Carbon-Monoxide-Questions-and-Answers — "[search excerpt] If you suspect CO poisoning, get outside to fresh air immediately, and then call 911 ... DO NOT reenter the premises until the emergency services responders have given you permission."</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -23894,7 +23921,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED — BLOCKING</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -24261,7 +24288,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>(not retrieved)</t>
+          <t>(not retrieved) · VERIFIED 2026-10-14 by Claude cloud session via official-domain web search (excerpts; confirm live wording at QA F-03): https://www.ready.gov/power-outages — "[search excerpt] gas stations rely on electricity to power their pumps; FCC NRIC 2003 blackout review: many cell towers had only 2-4 hours of backup battery power"</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -24271,12 +24298,12 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Backup durations vary widely</t>
+          <t>Historical figures (2003); no hour numbers on screen</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Avoid specific hours</t>
+          <t>"Phone towers run on backup power. Gas pumps need electricity."</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -24286,7 +24313,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED — BLOCKING if stated</t>
+          <t>QUALIFIED</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -24709,7 +24736,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>(not retrieved; e.g. British Antarctic Survey / NSF)</t>
+          <t>(not retrieved; e.g. British Antarctic Survey / NSF) · VERIFIED 2026-10-14 by Claude cloud session via official-domain web search (excerpts; confirm live wording at QA F-03): https://www.usap.gov/aboutthecontinent/ — "[search excerpt] the average monthly winter temperature is about −76°F [South Pole]; British Antarctic Survey: mean winter temperature of -59 C"</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -24719,7 +24746,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Coastal stations are milder</t>
+          <t>The −41 °C station readout is well within an inland winter range</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -24734,7 +24761,7 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED — BLOCKING if a number is shown</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -24933,7 +24960,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>NOAA (not retrieved)</t>
+          <t>NOAA (not retrieved) · VERIFIED 2026-10-14 by Claude cloud session via official-domain web search (excerpts; confirm live wording at QA F-03): https://www.noaa.gov/jetstream/ocean/rip-currents — "[search excerpt] a channel of churning, choppy water; a notable difference in water color; a line of foam, seaweed, or debris moving steadily seaward; a break in the incoming wave pattern"</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -24958,7 +24985,7 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED — BLOCKING if shown</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -24989,7 +25016,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>NASA / ESA (not retrieved)</t>
+          <t>NASA / ESA (not retrieved) · VERIFIED 2026-10-14 by Claude cloud session via official-domain web search (excerpts; confirm live wording at QA F-03): https://www.esa.int/ESA_Multimedia/Images/2023/02/Chelyabinsk_a_decade_on_the_Sun_s_invisible_asteroids — "the shockwave reached the ground damaging thousands of buildings, breaking windows and injuring roughly 1500 people from flying shards of glass (NASA: About two minutes later, the shock wave reached the ground; ESA planetary-defence guidance: move away from windows and glass and stay indoors)"</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -24999,7 +25026,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Injury counts differ by source (about 1,500 to 1,600): say 'most people hurt', no number</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -25014,7 +25041,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED — BLOCKING</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -25045,7 +25072,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>IMO / American Meteor Society / NASA (not retrieved)</t>
+          <t>IMO / American Meteor Society / NASA (not retrieved) · VERIFIED 2026-10-14 by Claude cloud session via official-domain web search (excerpts; confirm live wording at QA F-03): https://science.nasa.gov/solar-system/meteors-meteorites/leonids/ — "[search excerpt] activity Nov. 6 to Nov. 30, 2026, with a peak night of Nov. 16–17; AMS FAQ: meteor showers pose no meaningful danger to observers on the ground"</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -25055,7 +25082,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Must not imply the Leonids cause airbursts</t>
+          <t>Peak night 16–17 Nov (NASA) or 17–18 Nov (US Eastern, timeanddate): say 'this week' on screen</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -25070,7 +25097,7 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED — BLOCKING</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -25213,7 +25240,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>NOAA SWPC; NASA; Hydro-Québec (not retrieved)</t>
+          <t>NOAA SWPC; NASA; Hydro-Québec (not retrieved) · VERIFIED 2026-10-14 by Claude cloud session via official-domain web search (excerpts; confirm live wording at QA F-03): https://swpc.noaa.gov/noaa-space-weather-scales — "[search excerpt] G5 Extreme: some grid systems may experience complete collapse or blackouts. Transformers may experience damage. (NOAA: March 1989, Quebec went dark for 9 hours; Carrington 1859 overloaded telegraph lines)"</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -25223,12 +25250,12 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Impacts uncertain; avoid apocalyptic certainty</t>
+          <t>Quebec outage length differs (9 h NOAA vs 12 h NASA): say 'for hours'. Don't claim May 2024 was the first G5 since 2003. A transformer 'hum' is not sourced and must not be stated as fact</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>"In 1989, a solar storm blacked out Quebec for hours."</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -25238,7 +25265,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED — BLOCKING</t>
+          <t>QUALIFIED</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -25437,7 +25464,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>MN DNR ice thickness guidelines (not retrieved)</t>
+          <t>MN DNR ice thickness guidelines (not retrieved) · VERIFIED 2026-10-14 by Claude cloud session via official-domain web search (excerpts; confirm live wording at QA F-03): https://www.dnr.state.mn.us/safety/ice/thickness.html — "Wait for at least 4 inches of solid, clear ice. (white ice is about half as strong; double the guidelines)"</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -25447,22 +25474,22 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
+          <t>New clear ice only; Minnesota DNR guideline</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>"Four inches of new clear ice, minimum."</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED — BLOCKING if a number is shown</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -25493,7 +25520,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>CAL FIRE / IAFC Ready Set Go; NFPA Firewise (not retrieved)</t>
+          <t>CAL FIRE / IAFC Ready Set Go; NFPA Firewise (not retrieved) · VERIFIED 2026-10-14 by Claude cloud session via official-domain web search (excerpts; confirm live wording at QA F-03): https://www.nfpa.org/en/education-and-research/wildfire/preparing-homes-for-wildfire — "Embers are burning pieces of airborne wood and/or vegetation that can be carried more than a mile through the wind. (Ready.gov wildfires: evacuate immediately if authorities tell you to do so; USFA checklist: leaving early is wise if you are concerned)"</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -25508,17 +25535,17 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
+          <t>REAL RULE: "Wildfire: leave as soon as you're told to. Sooner if you feel unsafe."</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H57" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED — BLOCKING</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
@@ -25549,7 +25576,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Brugger/Haegeli survival-curve research; avalanche.org (not retrieved)</t>
+          <t>Brugger/Haegeli survival-curve research; avalanche.org (not retrieved) · VERIFIED 2026-10-14 by Claude cloud session via official-domain web search (excerpts; confirm live wording at QA F-03): https://pmc.ncbi.nlm.nih.gov/articles/PMC8507645/ — "[search excerpt] survival of more than 90% in the first 15 to 20 minutes of burial, followed by a steep decline in survival to 35% from 20 to 35 minutes; the likelihood of survival can be four times higher if the victim is rescued by uninjured companions compared to organized rescue (also CMAJ 183(7):E366; avalanche.org companion rescue)"</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -25559,22 +25586,22 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
+          <t>Survival curves vary by region: say 'survival drops fast after the first 15 minutes or so'; no exact cliff on screen</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>REAL RULE: "Avalanche: your partners are the rescue team. Speed is everything."</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED — BLOCKING</t>
+          <t>QUALIFIED</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -25605,7 +25632,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>NFPA; USFA; UL (not retrieved)</t>
+          <t>NFPA; USFA; UL (not retrieved) · VERIFIED 2026-10-14 by Claude cloud session via official-domain web search (excerpts; confirm live wording at QA F-03): https://www.usfa.fema.gov/statistics/reports/fire-causes/snapshot-thanksgiving.html — "[search excerpt] cooking fires in residential buildings occurred more often on Thanksgiving Day than any other day of the year; NFPA: never pour water on a cooking pan grease fire; smother with a lid and turn off the heat; turkey fryers outdoors away from the house, turkey fully thawed"</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -25615,22 +25642,22 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
+          <t>NFPA also states oil-based consumer turkey fryers are not suitable for safe use: the episode must not present frying as safe if done right (description note)</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>REAL RULE: "Grease fire? Never water. Lid on, heat off."</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G59" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H59" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED — BLOCKING</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
@@ -25661,7 +25688,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>G. Keith Still crowd science; agency guidance (not retrieved)</t>
+          <t>G. Keith Still crowd science; agency guidance (not retrieved) · VERIFIED 2026-10-14 by Claude cloud session via official-domain web search (excerpts; confirm live wording at QA F-03): https://theconversation.com/ten-tips-for-surviving-a-crowd-crush-112169 — "[search excerpt, crowd-safety researchers] fold your arms up in front of you like a boxer ... move away from any walls, pillars and fences ... move toward where the crowd thins out; the vast majority of deaths are caused by asphyxiation"</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -25671,12 +25698,12 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Sensitive topic</t>
+          <t>Expert (academic) guidance, not an agency standard. 'Move diagonally' is NOT supported: say 'toward where the crowd thins'. No density numbers. Sensitivity review still required</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>REAL RULE: "Crowd surge? Stay on your feet. Arms up to protect your chest."</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -25686,7 +25713,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED — BLOCKING</t>
+          <t>QUALIFIED</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
@@ -25717,7 +25744,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>NWS winter safety; Ready.gov winter weather (not retrieved)</t>
+          <t>NWS winter safety; Ready.gov winter weather (not retrieved) · VERIFIED 2026-10-14 by Claude cloud session via official-domain web search (excerpts; confirm live wording at QA F-03): https://www.weather.gov/media/ddc/NewsletterFall2009.pdf — "Run the motor about 10 minutes each hour for heat, but keep the window cracked and the exhaust pipe clear to prevent carbon monoxide poisoning. (NWS: If you leave your vehicle, you will become disoriented quickly in wind-driven snow and cold.)"</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -25732,17 +25759,17 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
+          <t>REAL RULE: "Stranded in snow? Stay with the car. Keep the tailpipe clear."</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED — BLOCKING</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">

</xml_diff>